<commit_message>
Updated reports and graphics (ongoing)
</commit_message>
<xml_diff>
--- a/reports/Angola_1.1_trade_balance_2003-2023.xlsx
+++ b/reports/Angola_1.1_trade_balance_2003-2023.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jrc/develop/cipf-comtrade/reports/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D38E4327-0300-9341-B306-671BFD5A1207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="20920" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -115,8 +121,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,13 +185,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -223,7 +237,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -257,6 +271,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -291,9 +306,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -466,11 +482,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="11" width="16.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -505,58 +524,58 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C2">
-        <v>4431063866.318</v>
+        <v>4431063866.3179998</v>
       </c>
       <c r="E2">
-        <v>9322134085.353001</v>
+        <v>9322134085.3530006</v>
       </c>
       <c r="G2">
-        <v>9322134085.353001</v>
+        <v>9322134085.3530006</v>
       </c>
       <c r="I2">
-        <v>9322134085.353001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>9322134085.3530006</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C3">
-        <v>6674906901.496</v>
+        <v>6674906901.4960003</v>
       </c>
       <c r="E3">
-        <v>12774810411.911</v>
+        <v>12774810411.910999</v>
       </c>
       <c r="G3">
-        <v>12774810411.911</v>
+        <v>12774810411.910999</v>
       </c>
       <c r="I3">
-        <v>12774810411.911</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+        <v>12774810411.910999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C4">
-        <v>7767184001.864</v>
+        <v>7767184001.8640003</v>
       </c>
       <c r="E4">
-        <v>22086367001.779</v>
+        <v>22086367001.778999</v>
       </c>
       <c r="G4">
-        <v>22086367001.779</v>
+        <v>22086367001.778999</v>
       </c>
       <c r="I4">
-        <v>22086367001.779</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+        <v>22086367001.778999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -564,16 +583,16 @@
         <v>10636294703.972</v>
       </c>
       <c r="E5">
-        <v>32047827417.37</v>
+        <v>32047827417.369999</v>
       </c>
       <c r="G5">
-        <v>32047827417.37</v>
+        <v>32047827417.369999</v>
       </c>
       <c r="I5">
-        <v>32047827417.37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+        <v>32047827417.369999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -581,13 +600,13 @@
         <v>11094843413</v>
       </c>
       <c r="C6">
-        <v>12662439392.449</v>
+        <v>12662439392.448999</v>
       </c>
       <c r="D6">
         <v>44177783071</v>
       </c>
       <c r="E6">
-        <v>41711887538.549</v>
+        <v>41711887538.549004</v>
       </c>
       <c r="F6">
         <v>33082939658</v>
@@ -599,33 +618,33 @@
         <v>55272626484</v>
       </c>
       <c r="I6">
-        <v>52806730951.549</v>
+        <v>52806730951.549004</v>
       </c>
       <c r="J6">
-        <v>0.8762011070012461</v>
+        <v>0.87620110700124609</v>
       </c>
       <c r="K6">
         <v>1.059117332682969</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C7">
-        <v>20453103082.927</v>
+        <v>20453103082.926998</v>
       </c>
       <c r="E7">
-        <v>67748978154.391</v>
+        <v>67748978154.390999</v>
       </c>
       <c r="G7">
-        <v>67748978154.391</v>
+        <v>67748978154.390999</v>
       </c>
       <c r="I7">
-        <v>67748978154.391</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+        <v>67748978154.390999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -639,28 +658,28 @@
         <v>40639411732</v>
       </c>
       <c r="E8">
-        <v>39936869089.036</v>
+        <v>39936869089.036003</v>
       </c>
       <c r="F8">
         <v>16720557371</v>
       </c>
       <c r="G8">
-        <v>16018014728.036</v>
+        <v>16018014728.035999</v>
       </c>
       <c r="H8">
         <v>64558266093</v>
       </c>
       <c r="I8">
-        <v>63855723450.036</v>
+        <v>63855723450.036003</v>
       </c>
       <c r="J8">
         <v>1.34086603288823</v>
       </c>
       <c r="K8">
-        <v>1.017591329991285</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
+        <v>1.0175913299912851</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -674,28 +693,28 @@
         <v>52612114761</v>
       </c>
       <c r="E9">
-        <v>53460941627.269</v>
+        <v>53460941627.268997</v>
       </c>
       <c r="F9">
         <v>34468845853</v>
       </c>
       <c r="G9">
-        <v>35317672719.269</v>
+        <v>35317672719.268997</v>
       </c>
       <c r="H9">
         <v>70755383669</v>
       </c>
       <c r="I9">
-        <v>71604210535.26901</v>
+        <v>71604210535.269012</v>
       </c>
       <c r="J9">
-        <v>1.143219320628997</v>
+        <v>1.1432193206289969</v>
       </c>
       <c r="K9">
-        <v>0.9841224856796005</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+        <v>0.98412248567960048</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -709,28 +728,28 @@
         <v>66427390220</v>
       </c>
       <c r="E10">
-        <v>66207593128.22</v>
+        <v>66207593128.220001</v>
       </c>
       <c r="F10">
         <v>45636394181</v>
       </c>
       <c r="G10">
-        <v>45416597089.22</v>
+        <v>45416597089.220001</v>
       </c>
       <c r="H10">
         <v>87218386259</v>
       </c>
       <c r="I10">
-        <v>86998589167.22</v>
+        <v>86998589167.220001</v>
       </c>
       <c r="J10">
-        <v>1.134053357395156</v>
+        <v>1.1340533573951559</v>
       </c>
       <c r="K10">
-        <v>1.00331981697861</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+        <v>1.0033198169786099</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -744,13 +763,13 @@
         <v>70863076413</v>
       </c>
       <c r="E11">
-        <v>75489311613.616</v>
+        <v>75489311613.615997</v>
       </c>
       <c r="F11">
         <v>42140092349</v>
       </c>
       <c r="G11">
-        <v>46766327549.616</v>
+        <v>46766327549.615997</v>
       </c>
       <c r="H11">
         <v>99586060477</v>
@@ -759,13 +778,13 @@
         <v>104212295677.616</v>
       </c>
       <c r="J11">
-        <v>1.298946451386444</v>
+        <v>1.2989464513864439</v>
       </c>
       <c r="K11">
-        <v>0.9387166858230885</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
+        <v>0.93871668582308854</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -773,7 +792,7 @@
         <v>26756062991</v>
       </c>
       <c r="C12">
-        <v>24445948776.321</v>
+        <v>24445948776.320999</v>
       </c>
       <c r="D12">
         <v>67712526547</v>
@@ -794,13 +813,13 @@
         <v>99062735065.612</v>
       </c>
       <c r="J12">
-        <v>1.094498856878758</v>
+        <v>1.0944988568787579</v>
       </c>
       <c r="K12">
-        <v>0.9364630483495163</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+        <v>0.93646304834951632</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -808,19 +827,19 @@
         <v>28753499329</v>
       </c>
       <c r="C13">
-        <v>28410762457.261</v>
+        <v>28410762457.261002</v>
       </c>
       <c r="D13">
         <v>58672369190</v>
       </c>
       <c r="E13">
-        <v>64697442327.26</v>
+        <v>64697442327.260002</v>
       </c>
       <c r="F13">
         <v>29918869861</v>
       </c>
       <c r="G13">
-        <v>35943942998.26</v>
+        <v>35943942998.260002</v>
       </c>
       <c r="H13">
         <v>87425868519</v>
@@ -832,27 +851,27 @@
         <v>1.012063628079485</v>
       </c>
       <c r="K13">
-        <v>0.9068730861602954</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
+        <v>0.90687308616029538</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B14">
-        <v>21549256530.51</v>
+        <v>21549256530.509998</v>
       </c>
       <c r="C14">
-        <v>18527008742.047</v>
+        <v>18527008742.047001</v>
       </c>
       <c r="D14">
-        <v>33924937478.31</v>
+        <v>33924937478.310001</v>
       </c>
       <c r="E14">
-        <v>36838371233.673</v>
+        <v>36838371233.672997</v>
       </c>
       <c r="F14">
-        <v>12375680947.8</v>
+        <v>12375680947.799999</v>
       </c>
       <c r="G14">
         <v>15289114703.16301</v>
@@ -861,27 +880,27 @@
         <v>55474194008.82</v>
       </c>
       <c r="I14">
-        <v>58387627764.183</v>
+        <v>58387627764.182999</v>
       </c>
       <c r="J14">
-        <v>1.163126591590795</v>
+        <v>1.1631265915907949</v>
       </c>
       <c r="K14">
         <v>0.9209130681461859</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B15">
-        <v>14347710497.8</v>
+        <v>14347710497.799999</v>
       </c>
       <c r="C15">
-        <v>11654615725.7</v>
+        <v>11654615725.700001</v>
       </c>
       <c r="D15">
-        <v>28057499522.39</v>
+        <v>28057499522.389999</v>
       </c>
       <c r="E15">
         <v>28307515856.945</v>
@@ -893,19 +912,19 @@
         <v>13959805359.145</v>
       </c>
       <c r="H15">
-        <v>42405210020.19</v>
+        <v>42405210020.190002</v>
       </c>
       <c r="I15">
-        <v>42655226354.745</v>
+        <v>42655226354.745003</v>
       </c>
       <c r="J15">
         <v>1.231075381246707</v>
       </c>
       <c r="K15">
-        <v>0.9911678461713672</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
+        <v>0.99116784617136722</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>25</v>
       </c>
@@ -913,45 +932,45 @@
         <v>15462313478.23</v>
       </c>
       <c r="C16">
-        <v>11876470470.501</v>
+        <v>11876470470.500999</v>
       </c>
       <c r="D16">
-        <v>34904881109.37</v>
+        <v>34904881109.370003</v>
       </c>
       <c r="E16">
-        <v>36707626909.324</v>
+        <v>36707626909.323997</v>
       </c>
       <c r="F16">
-        <v>19442567631.14</v>
+        <v>19442567631.139999</v>
       </c>
       <c r="G16">
-        <v>21245313431.094</v>
+        <v>21245313431.094002</v>
       </c>
       <c r="H16">
-        <v>50367194587.60001</v>
+        <v>50367194587.600014</v>
       </c>
       <c r="I16">
-        <v>52169940387.554</v>
+        <v>52169940387.554001</v>
       </c>
       <c r="J16">
-        <v>1.301928339453677</v>
+        <v>1.3019283394536769</v>
       </c>
       <c r="K16">
-        <v>0.9508890671574282</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
+        <v>0.95088906715742816</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B17">
-        <v>16006910579.064</v>
+        <v>16006910579.063999</v>
       </c>
       <c r="C17">
         <v>10345721895.857</v>
       </c>
       <c r="D17">
-        <v>40664718814.96</v>
+        <v>40664718814.959999</v>
       </c>
       <c r="E17">
         <v>44190259295.527</v>
@@ -960,68 +979,68 @@
         <v>24657808235.896</v>
       </c>
       <c r="G17">
-        <v>28183348716.463</v>
+        <v>28183348716.463001</v>
       </c>
       <c r="H17">
-        <v>56671629394.024</v>
+        <v>56671629394.024002</v>
       </c>
       <c r="I17">
-        <v>60197169874.591</v>
+        <v>60197169874.591003</v>
       </c>
       <c r="J17">
         <v>1.54720093389269</v>
       </c>
       <c r="K17">
-        <v>0.9202190587525279</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+        <v>0.92021905875252785</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B18">
-        <v>13961640425.765</v>
+        <v>13961640425.764999</v>
       </c>
       <c r="C18">
-        <v>9481649454.854</v>
+        <v>9481649454.8540001</v>
       </c>
       <c r="D18">
-        <v>35432454858.832</v>
+        <v>35432454858.832001</v>
       </c>
       <c r="E18">
-        <v>37542311664.656</v>
+        <v>37542311664.655998</v>
       </c>
       <c r="F18">
-        <v>21470814433.067</v>
+        <v>21470814433.067001</v>
       </c>
       <c r="G18">
-        <v>23580671238.891</v>
+        <v>23580671238.890999</v>
       </c>
       <c r="H18">
         <v>49394095284.597</v>
       </c>
       <c r="I18">
-        <v>51503952090.421</v>
+        <v>51503952090.420998</v>
       </c>
       <c r="J18">
         <v>1.472490677096012</v>
       </c>
       <c r="K18">
-        <v>0.9438005622916846</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
+        <v>0.94380056229168463</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B19">
-        <v>9337925708.641001</v>
+        <v>9337925708.6410007</v>
       </c>
       <c r="C19">
-        <v>7579164285.011</v>
+        <v>7579164285.0109997</v>
       </c>
       <c r="D19">
-        <v>22134505473.377</v>
+        <v>22134505473.376999</v>
       </c>
       <c r="E19">
         <v>24012461247.855</v>
@@ -1030,22 +1049,22 @@
         <v>12796579764.736</v>
       </c>
       <c r="G19">
-        <v>14674535539.214</v>
+        <v>14674535539.214001</v>
       </c>
       <c r="H19">
-        <v>31472431182.018</v>
+        <v>31472431182.018002</v>
       </c>
       <c r="I19">
-        <v>33350386956.496</v>
+        <v>33350386956.495998</v>
       </c>
       <c r="J19">
-        <v>1.23205215740055</v>
+        <v>1.2320521574005501</v>
       </c>
       <c r="K19">
-        <v>0.9217924495496789</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11">
+        <v>0.92179244954967887</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
@@ -1056,66 +1075,66 @@
         <v>9449572419.052</v>
       </c>
       <c r="D20">
-        <v>34472161956.832</v>
+        <v>34472161956.832001</v>
       </c>
       <c r="E20">
-        <v>33645511738.133</v>
+        <v>33645511738.132999</v>
       </c>
       <c r="F20">
-        <v>23093234036.131</v>
+        <v>23093234036.131001</v>
       </c>
       <c r="G20">
-        <v>22266583817.432</v>
+        <v>22266583817.431999</v>
       </c>
       <c r="H20">
-        <v>45851089877.533</v>
+        <v>45851089877.532997</v>
       </c>
       <c r="I20">
         <v>45024439658.834</v>
       </c>
       <c r="J20">
-        <v>1.204173841533727</v>
+        <v>1.2041738415337271</v>
       </c>
       <c r="K20">
-        <v>1.024569405427176</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
+        <v>1.0245694054271759</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B21">
-        <v>17802935241.948</v>
+        <v>17802935241.948002</v>
       </c>
       <c r="C21">
         <v>14267672182.795</v>
       </c>
       <c r="D21">
-        <v>51274951711.647</v>
+        <v>51274951711.647003</v>
       </c>
       <c r="E21">
-        <v>52943571614.454</v>
+        <v>52943571614.454002</v>
       </c>
       <c r="F21">
-        <v>33472016469.699</v>
+        <v>33472016469.699001</v>
       </c>
       <c r="G21">
-        <v>35140636372.506</v>
+        <v>35140636372.505997</v>
       </c>
       <c r="H21">
-        <v>69077886953.595</v>
+        <v>69077886953.595001</v>
       </c>
       <c r="I21">
-        <v>70746506856.40201</v>
+        <v>70746506856.402008</v>
       </c>
       <c r="J21">
-        <v>1.247781348902597</v>
+        <v>1.2477813489025971</v>
       </c>
       <c r="K21">
-        <v>0.9684830499355382</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
+        <v>0.96848304993553824</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -1123,13 +1142,13 @@
         <v>10812915513.618</v>
       </c>
       <c r="E22">
-        <v>35312785387.256</v>
+        <v>35312785387.255997</v>
       </c>
       <c r="G22">
-        <v>35312785387.256</v>
+        <v>35312785387.255997</v>
       </c>
       <c r="I22">
-        <v>35312785387.256</v>
+        <v>35312785387.255997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>